<commit_message>
scan: seg0 2026-10-14 00:59 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-10-13.xlsx
+++ b/output/full_scan/batch_seq1_2026-10-13.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>77.25136717259093</v>
+        <v>77.2513672842158</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>45.40178765697296</v>
+        <v>45.40178771432889</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>5.635494940696374</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.1784221636264444</v>
+        <v>0.1784221635423215</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>61.94564589847283</v>
+        <v>61.94564597270626</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>15.50021523724256</v>
+        <v>15.50021531377154</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.725323563765558</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.3473827985395464</v>
+        <v>0.3473827984914728</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>69.02595172139732</v>
+        <v>69.02595205582955</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>34.32862702328924</v>
+        <v>34.32862712125957</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.15578531229981</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.062242067753096</v>
+        <v>0.0622420676569571</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>74.69552887928184</v>
+        <v>74.69552892528351</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>43.49633869608985</v>
+        <v>43.4963387808661</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>3.69927634537917</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.7456241558934193</v>
+        <v>0.7456241557080578</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>67.57421610624439</v>
+        <v>67.5742160919159</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>25.15711752013359</v>
+        <v>25.15711759636538</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>1.088726766154096</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.0877874146619569</v>
+        <v>0.08778741464993869</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>75.40267347583331</v>
+        <v>75.40267358356637</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>32.35090397146166</v>
+        <v>32.35090401999101</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.666410560283429</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.2115806917490387</v>
+        <v>0.2115806917009687</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>81.15282131463715</v>
+        <v>81.15282135582405</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>26.93604160297448</v>
+        <v>26.93604165987573</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>4.608569857969152</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.1416060426132359</v>
+        <v>0.1416060426012196</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68.55193308227575</v>
+        <v>68.55193316140817</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>33.50635472629729</v>
+        <v>33.50635494460989</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>2.739353102159029</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-0.3168122073225206</v>
+        <v>-0.3168122076589923</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1082.793183700185</v>
+        <v>1082.793183700186</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>14.5</v>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>59.95743089188638</v>
+        <v>59.95743110771149</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>36.25851962025834</v>
+        <v>36.2585196872342</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.061283189684504</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.0475063474120374</v>
+        <v>0.0475063473519501</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>63.17633551457691</v>
+        <v>63.17633561811328</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>9.677046768699356</v>
+        <v>9.677046771492044</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.622238217488491</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.0542644077923092</v>
+        <v>0.0542644077682759</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>67.55103161507452</v>
+        <v>67.55103182284425</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>26.17670917908868</v>
+        <v>26.17670930386195</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.957035402152703</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.1181271769789331</v>
+        <v>0.1181271769188464</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>64.18923971894839</v>
+        <v>64.18924000494685</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>19.38722474736554</v>
+        <v>19.38722488802518</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>6.915088744406413</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.4117842174186231</v>
+        <v>0.4117842169379343</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.40748561280284</v>
+        <v>60.40748582749016</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>37.70655834267362</v>
+        <v>37.7065585029588</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>2.396092540794917</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.0442684371103843</v>
+        <v>0.0442684370382811</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>82.91681945860735</v>
+        <v>82.91681957451678</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>65.31394710094477</v>
+        <v>65.31394715069605</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>3.002685624105092</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>1.233388988989677</v>
+        <v>1.23338898846092</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>66.66826870511036</v>
+        <v>66.66826897667954</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>35.16755227045272</v>
+        <v>35.1675523913403</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>2.696970801573137</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.1040944566583568</v>
+        <v>0.1040944565622185</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>978.2641554258956</v>
+        <v>978.2641554258958</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>77.8</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>68.28382622743042</v>
+        <v>68.28382634128106</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>33.66667995673609</v>
+        <v>33.66668014102648</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.708777511165783</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.8286504395661289</v>
+        <v>0.8286504393498211</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>67.15021898571001</v>
+        <v>67.1502189922634</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>14.35456488597402</v>
+        <v>14.35456488606698</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>4.384656289391733</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>75.73115046661636</v>
+        <v>75.7311504856342</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>41.83553749255632</v>
+        <v>41.83553761337422</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.596911432692943</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>6.050393446263982</v>
+        <v>6.05039344592748</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>60.41192224638436</v>
+        <v>60.41192240220445</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>41.3818043123162</v>
+        <v>41.38180460494224</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.6053970327402267</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.0015633825410407</v>
+        <v>0.0015633825025861</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>78.42986078160105</v>
+        <v>78.42986088299962</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>34.49243377997269</v>
+        <v>34.49243389299969</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>2.47442323923965</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.595154478750572</v>
+        <v>1.595154478486195</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>900.6293531271058</v>
+        <v>900.6293531271057</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>10.2</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>69.40684407770888</v>
+        <v>69.40684426685036</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>45.3632907094383</v>
+        <v>45.36329088609075</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>2.372951981940106</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.1115132026257788</v>
+        <v>0.1115132025488668</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>63.9279785823236</v>
+        <v>63.92797867851662</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>28.10940447376172</v>
+        <v>28.10940448780892</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.018261009891605</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>2.199761974133353</v>
+        <v>2.199761974493859</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>837.6158033250701</v>
+        <v>837.6158033250633</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>27.1</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>63.13931221675438</v>
+        <v>63.13931253649236</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>31.140925316078</v>
+        <v>31.1409252417987</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>3.437442641329018</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.1684973324457733</v>
+        <v>0.1684973322655122</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>819.5120323020371</v>
+        <v>819.5120323020369</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>950</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>58.58408037961539</v>
+        <v>58.58408044093908</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>48.88415654314819</v>
+        <v>48.88415657429803</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.8869954361000967</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-3.734634581026029</v>
+        <v>-3.734634582227713</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>804.8010699493809</v>
+        <v>804.801069949381</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>25.75</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>57.57114079821438</v>
+        <v>57.57114105925962</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>22.62362433225821</v>
+        <v>22.62362486889057</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.9433488209772336</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.1548586844816764</v>
+        <v>0.1548586841572087</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>59.54847058617513</v>
+        <v>59.54847064780749</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>20.18126697274996</v>
+        <v>20.1812669838304</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.5791991627916815</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.0921648825771476</v>
+        <v>0.0921648825531127</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>60.42226549573271</v>
+        <v>60.42226546479387</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>42.42347258508071</v>
+        <v>42.42347272978403</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.271642256817265</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.1373194486350897</v>
+        <v>0.1373194486471053</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>53.49370382701221</v>
+        <v>53.49370405970699</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>24.5823806839907</v>
+        <v>24.58238079973406</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>4.324148543404498</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.0412308379923058</v>
+        <v>0.0412308379081826</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>55.59947144333827</v>
+        <v>55.59947160472189</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>18.69837912111178</v>
+        <v>18.69837895587853</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.030672807997268</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.0025114110331022</v>
+        <v>0.0025114109970517</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>59.97653692754377</v>
+        <v>59.97653691322182</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>23.84602674964255</v>
+        <v>23.84602678190047</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.5257438999124915</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.0583364277814291</v>
+        <v>0.0583364277694118</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>82.15531101728403</v>
+        <v>82.15531103711321</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>52.20993766701562</v>
+        <v>52.20993768090801</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.977430807479854</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.4767742181334369</v>
+        <v>0.4767742181094083</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>55.09597945345751</v>
+        <v>55.09597948219395</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>13.29042260406058</v>
+        <v>13.29042260758557</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.5625435623911625</v>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>711.9483391239023</v>
+        <v>711.9483391239022</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>165.5</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>48.24065855384465</v>
+        <v>48.24065847747566</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>9.65523463607262</v>
+        <v>9.655234744064812</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.346781300756536</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.0098343946694934</v>
+        <v>0.0098343945493184</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>711.0469166818566</v>
+        <v>711.0469166818567</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>17.7</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>56.14718960908284</v>
+        <v>56.14718971769407</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>17.49280971082556</v>
+        <v>17.49280978109336</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>2.626694956659282</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.0200027304263359</v>
+        <v>0.0200027303902845</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>57.40150218415286</v>
+        <v>57.40150230817736</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>38.41468524824064</v>
+        <v>38.4146854394972</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.99216670119149</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.0437793422870865</v>
+        <v>0.0437793421188456</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>62.93885168534505</v>
+        <v>62.93885174864506</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>22.53751189871144</v>
+        <v>22.53751189620727</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>2.001418142233674</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.0971091878121642</v>
+        <v>0.09710918778812951</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>78.4461907543261</v>
+        <v>78.44619076725158</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>33.28490384637523</v>
+        <v>33.28490384456711</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>3.95880213884439</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.6134806961108197</v>
+        <v>0.6134806961588872</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>57.3928959372363</v>
+        <v>57.39289573186189</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>21.24371488435297</v>
+        <v>21.24371496946549</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>1.111159135755881</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0461351208628833</v>
+        <v>0.0461351208989361</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>65.31202788501619</v>
+        <v>65.3120281362109</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>37.49490227869739</v>
+        <v>37.49490237341369</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.9133143551510012</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>5.655750005796635</v>
+        <v>5.655750003393178</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>53.44221552257009</v>
+        <v>53.44221554532327</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>8.96780617604405</v>
+        <v>8.967806166519319</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.268365419773835</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>52.04011865050015</v>
+        <v>52.04011906395274</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>21.16506287899436</v>
+        <v>21.16506282636443</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.5047565838314416</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.0239844007073037</v>
+        <v>0.0239844006592359</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>652.7910785101552</v>
+        <v>652.7910785101551</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>25.65</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>50.90440188760744</v>
+        <v>50.90440202144528</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>30.62819813013251</v>
+        <v>30.62819837508109</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7313552939055872</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.0213403309634662</v>
+        <v>0.0213403308673307</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>52.16273023301447</v>
+        <v>52.16273038955582</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>7.954609472998486</v>
+        <v>7.954609394231862</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.9018867738094648</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.0189985494181025</v>
+        <v>0.0189985493580165</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>639.1523096271829</v>
+        <v>639.1523096271831</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>69.7</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.87354352198879</v>
+        <v>47.87354389228996</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>17.5398425771341</v>
+        <v>17.53984269058077</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8806263421136417</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.1869902831597879</v>
+        <v>0.186990283207856</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>49.12652013360925</v>
+        <v>49.12652061398998</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>17.46296453138977</v>
+        <v>17.46296457853835</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5848585516479576</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0016049024558471</v>
+        <v>0.001604902407778</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>52.2780003897832</v>
+        <v>52.27800047540494</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>35.44525151556736</v>
+        <v>35.44525153794611</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8982002362467871</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.035163862545743</v>
+        <v>0.0351638625553558</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>47.22566847692956</v>
+        <v>47.22566853080347</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>10.71768498927667</v>
+        <v>10.71768495694544</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.086640215191165</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>52.26196412592498</v>
+        <v>52.26196416910174</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>24.47402747764348</v>
+        <v>24.47402759557722</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>4.255715521416234</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.1815755529270438</v>
+        <v>0.181575552806871</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>49.13745656335959</v>
+        <v>49.13745671074668</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>21.60531933597661</v>
+        <v>21.60531947030831</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.5694446660154044</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.1017704892658628</v>
+        <v>0.101770489307054</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>591.4763210474495</v>
+        <v>591.4763210474496</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>198.5</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>48.90846070374804</v>
+        <v>48.90846082504435</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>10.25204267121491</v>
+        <v>10.25204277662115</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.685481512457879</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.5716997276157882</v>
+        <v>0.5716997266543957</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>49.83781135398485</v>
+        <v>49.83781165262384</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>13.82779323712085</v>
+        <v>13.82779330851253</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.569608726862702</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0006207036081275</v>
+        <v>0.0006207035961116</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>590.8689255232429</v>
+        <v>590.8689255232432</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>40.65</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.02472946865742</v>
+        <v>53.02472978908405</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>19.56826364309825</v>
+        <v>19.56826371978076</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.682862720811732</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0769082173645572</v>
+        <v>0.07690821718429409</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>580.6288928765966</v>
+        <v>580.6288928765965</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>9.66</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>58.98103784032958</v>
+        <v>58.98103786869987</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>26.5253155955928</v>
+        <v>26.52531579940522</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.5350162707557826</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.034057119708502</v>
+        <v>0.0340571197275721</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>573.6506062484436</v>
+        <v>573.6506062484438</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>88.59999999999999</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>52.83096810797067</v>
+        <v>52.83096813747378</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>8.273357015774005</v>
+        <v>8.273357283774125</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>2.714614555260498</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.5170556606354593</v>
+        <v>0.5170556600586358</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.37077099461531</v>
+        <v>44.37077104960229</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>42.73844857767856</v>
+        <v>42.73844856640098</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.9757975031834616</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.0434605526443789</v>
+        <v>0.0434605526323596</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>569.3671262248226</v>
+        <v>569.3671262248228</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>22.65</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>45.84320869231139</v>
+        <v>45.84320882758866</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>34.22786383049514</v>
+        <v>34.22786387778831</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.1875654132327991</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.447784577645443</v>
+        <v>-0.4477845779819291</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>45.80111853910257</v>
+        <v>45.80111856411043</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>9.063495508728151</v>
+        <v>9.063495525347896</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>1.140781884212775</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.0017225861956348</v>
+        <v>0.001722586123534</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>56.11432894783428</v>
+        <v>56.11432942805403</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>14.34957088472558</v>
+        <v>14.34957090346705</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.673233906335242</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.0451597773112254</v>
+        <v>0.0451597772751729</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>544.9507736740894</v>
+        <v>544.9507736740895</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>65.90000000000001</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>48.92356559922494</v>
+        <v>48.92356591649762</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>10.94551204046745</v>
+        <v>10.94551206560016</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.886753086531745</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.0060458298638239</v>
+        <v>-0.0060458301762753</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>544.6598138547126</v>
+        <v>544.6598138547125</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>6.16</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>35.24510092210177</v>
+        <v>35.2451010010156</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>27.05765896464596</v>
+        <v>27.0576590079042</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.245690382534761</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0029933161071957</v>
+        <v>0.0029933161023893</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>48.24980531792461</v>
+        <v>48.24980562636544</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>14.42157569145398</v>
+        <v>14.42157586575359</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>1.22298930420948</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.1772365614162808</v>
+        <v>0.1772365606952476</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>539.9350102235309</v>
+        <v>539.9350102235308</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>13.2</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>52.37299077713991</v>
+        <v>52.3729909518464</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>27.73328439220119</v>
+        <v>27.73328450309092</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.8369770514192852</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0143984457860973</v>
+        <v>0.0143984457620629</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>36.83797229186268</v>
+        <v>36.83797244861805</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>27.40509396450322</v>
+        <v>27.40509397217464</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1.688420708469331</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>50.45826142378254</v>
+        <v>50.45826145039513</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>16.47942357273131</v>
+        <v>16.47942360010482</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.8449660158004058</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.0371543674953591</v>
+        <v>0.0371543674833401</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>526.2664916367054</v>
+        <v>526.2664916367053</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>11.9</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>51.88877579087126</v>
+        <v>51.88877583332794</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>16.50707168992157</v>
+        <v>16.50707173988377</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5919701714185014</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.07297307733952681</v>
+        <v>0.07297307735154521</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3983,7 +3983,7 @@
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>518.9711011790652</v>
+        <v>518.971101179065</v>
       </c>
       <c r="E67" s="2" t="n">
         <v>9.94</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>41.84709446335125</v>
+        <v>41.84709480566458</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>24.32278650361575</v>
+        <v>24.32278652079026</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.9702850384859238</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0074938285411721</v>
+        <v>0.0074938284931013</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>515.1886711064177</v>
+        <v>515.1886711064178</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>100.5</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>45.94116461480552</v>
+        <v>45.94116476620233</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>17.17617335793501</v>
+        <v>17.17617346404936</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.6893185699147537</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.2018600997572666</v>
+        <v>0.2018600993726982</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>52.56863703973024</v>
+        <v>52.56863726272411</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>14.59974210517889</v>
+        <v>14.59974214735409</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.227782944451209</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.07436756358359541</v>
+        <v>0.0743675633913167</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>45.26086270413822</v>
+        <v>45.26086282710686</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>27.2589452567777</v>
+        <v>27.25894533903839</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5203789483485022</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.0448085288245587</v>
+        <v>0.0448085287043848</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>486.1706273595036</v>
+        <v>486.1706273595031</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>13.45</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>46.79083564634487</v>
+        <v>46.79083568455519</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>15.03901798921442</v>
+        <v>15.03901793347674</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.577341661157281</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.012601826203324</v>
+        <v>0.0126018261312215</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>483.06340974591</v>
+        <v>483.0634097459093</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>59.5</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>51.91986052638369</v>
+        <v>51.91986052780567</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>8.875302942368778</v>
+        <v>8.875302948677284</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>2.854581723606797</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.9718965825336084</v>
+        <v>0.9718965822451856</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4318,7 +4318,7 @@
         <v>44.65253099949515</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>29.70667157660049</v>
+        <v>29.70667160022498</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.7486269876362441</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.2922466361296991</v>
+        <v>0.2922466357691906</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>468.8881871729178</v>
+        <v>468.8881871729176</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>9.27</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>59.56258897867188</v>
+        <v>59.56258895985066</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.48458560920281</v>
+        <v>14.48458559910783</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>2.13395528063682</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.6473457506043407</v>
+        <v>0.6473457505923237</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>48.42739884957554</v>
+        <v>48.42739895289272</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>12.54709555097412</v>
+        <v>12.54709557894565</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.107644234917953</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>48.72838846329272</v>
+        <v>48.72838855316411</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>16.73758057888656</v>
+        <v>16.73758063175389</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.8349522992392877</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.1052173645843995</v>
+        <v>0.1052173644401905</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>47.58502941138827</v>
+        <v>47.58502945692852</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>12.84294432763175</v>
+        <v>12.8429443826501</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.5855125041102226</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0127627822761528</v>
+        <v>0.0127627822521184</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>42.87284047063187</v>
+        <v>42.87284058725467</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>23.07791769425328</v>
+        <v>23.07791773534921</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1.067282594740367</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.0205341340493729</v>
+        <v>0.0205341340373555</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>455.4536439589289</v>
+        <v>455.4536439589348</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>26.55</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>34.73758036980986</v>
+        <v>34.73757964131676</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>31.81086159282369</v>
+        <v>31.81086165400077</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.2391974036913388</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.1725426593696751</v>
+        <v>-0.1725426594658149</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>455.040997764909</v>
+        <v>455.0409977649091</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>13.1</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>32.69282113457639</v>
+        <v>32.69282127769927</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>44.62951946869273</v>
+        <v>44.6295192760231</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.966409152000298</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.008529417311505701</v>
+        <v>-0.0085294173595762</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>64.1088467104079</v>
+        <v>64.10884669483332</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>64.05604383926554</v>
+        <v>64.05604400760551</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.7057625900881044</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.1039006565367272</v>
+        <v>0.103900656577917</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>440.8998055653037</v>
+        <v>440.8998055653036</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>5.08</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>40.144084308171</v>
+        <v>40.14408434416138</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>10.69822958767191</v>
+        <v>10.69822961264718</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>2.132432500440351</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.0115004652401035</v>
+        <v>-0.0115004652304897</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>47.51342949438197</v>
+        <v>47.51342969029472</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>21.2841843728942</v>
+        <v>21.28418441986393</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.8031629422587004</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0240528491261258</v>
+        <v>0.0240528491357392</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>50.41717422995951</v>
+        <v>50.4171744440024</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>11.5029468730548</v>
+        <v>11.50294696256848</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.059678007633542</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.035064712256986</v>
+        <v>0.0350647121848847</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>46.622961154926</v>
+        <v>46.62296123441285</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.02500560440263</v>
+        <v>17.0250055720714</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.389060772269596</v>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>427.9700105611272</v>
+        <v>427.9700105611271</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>8.119999999999999</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>46.52834398383106</v>
+        <v>46.52834410092989</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.75734902899033</v>
+        <v>17.75734884389578</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>1.446476345327126</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.015963138190093</v>
+        <v>0.0159631381876896</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>418.9507109372331</v>
+        <v>418.9507109372332</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>7.28</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>51.26331338488176</v>
+        <v>51.26331228536413</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>8.127324479495162</v>
+        <v>8.127323963387511</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.7550463823643209</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.0107599948712221</v>
+        <v>0.0107599978515129</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>49.04857148300036</v>
+        <v>49.04857158306202</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>20.43502588358204</v>
+        <v>20.4350259309796</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.6442112655837693</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0265117166339561</v>
+        <v>0.0265117166219415</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>47.04865989772228</v>
+        <v>47.04865998495648</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>18.340309497874</v>
+        <v>18.340309500229</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.971002748620334</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.0026704944301223</v>
+        <v>-0.0026704944421402</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>47.29493671641709</v>
+        <v>47.29493673131381</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>13.54308428063721</v>
+        <v>13.54308425149713</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6246051551335929</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.1102384580878822</v>
+        <v>0.1102384580638513</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>399.9783702086634</v>
+        <v>399.9783702086636</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>77.09999999999999</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>27.2906419348019</v>
+        <v>27.29064114311518</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>20.25448787723728</v>
+        <v>20.25448785256152</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.653914710732782</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1481488820901084</v>
+        <v>-0.1481488823304688</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>399.5357057683343</v>
+        <v>399.5357057683345</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>18.85</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>21.90504514723935</v>
+        <v>21.90504531492965</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>46.59634119410801</v>
+        <v>46.5963412140897</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>1.317133432210509</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0409534467311394</v>
+        <v>-0.0409534468513148</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>398.7579097658023</v>
+        <v>398.757909765803</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>9.98</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>48.48223865148763</v>
+        <v>48.48223935368617</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.44158318204326</v>
+        <v>17.44158364235242</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.8228372949429924</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.0033027788201057</v>
+        <v>0.0033027787119497</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,7 +5428,7 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>46.27002547411166</v>
+        <v>46.27002553260185</v>
       </c>
       <c r="I94" s="2" t="n">
         <v>17.42658713597072</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>45.04820602254077</v>
+        <v>45.04820613642006</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.92029221905501</v>
+        <v>16.92029231602784</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.6175280542526753</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0943126445822302</v>
+        <v>0.0943126444981105</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>48.98032025038376</v>
+        <v>48.98032044677205</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>35.88411752135455</v>
+        <v>35.88411746783687</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.6312603136259872</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0140959261658827</v>
+        <v>0.0140959261057949</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>38.84495906771252</v>
+        <v>38.84495906438342</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>13.6931147451546</v>
+        <v>13.69311482264859</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>3.231246784561097</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>51.47987310432107</v>
+        <v>51.47987310351783</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.47921038778213</v>
+        <v>19.47921035093741</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>2.535360333155022</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.192994046010048</v>
+        <v>-0.1929940459980264</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>48.74843417822512</v>
+        <v>48.74843425197978</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.83079414912727</v>
+        <v>16.83079409400038</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4307374331933649</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0133633035871784</v>
+        <v>0.0133633035751611</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>373.1375761887648</v>
+        <v>373.1375761887646</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>21.5</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>30.64022656105003</v>
+        <v>30.64022672192221</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>22.48981703912456</v>
+        <v>22.48981709714449</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.7214573609786515</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.07405338597570869</v>
+        <v>-0.0740533861199161</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.76572265538923</v>
+        <v>44.76572279061546</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>22.30464645291755</v>
+        <v>22.30464639850929</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.8441562046763346</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0236858247929727</v>
+        <v>0.0236858247809557</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>371.0407959248084</v>
+        <v>371.0407959248082</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>42.9</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>45.74626911737831</v>
+        <v>45.7462691429625</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>9.920394720966536</v>
+        <v>9.920394720966533</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.569970708934914</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>0.0226161380332911</v>
+        <v>0.02261613794917</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         <v>51.93021843002738</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>8.378348004397461</v>
+        <v>8.378347994610847</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>1.779383574071298</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>49.47600485735217</v>
+        <v>49.47600514289796</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>8.973912576928555</v>
+        <v>8.973912728297131</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.618895569477193</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.0030155558172226</v>
+        <v>-0.0030155559253772</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6014,7 +6014,7 @@
         <v>38.96278008861416</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>22.04760672365874</v>
+        <v>22.04760675037804</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.239246739320049</v>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>360.3127162391007</v>
+        <v>360.3127162391008</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>32.25</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>38.89133250045018</v>
+        <v>38.89133290333211</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>10.51431342469636</v>
+        <v>10.51431363429914</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.8286719326622591</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0204505691768314</v>
+        <v>-0.0204505693090211</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>344.7105385829151</v>
+        <v>344.7105385829141</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>61.6</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>49.178502141422</v>
+        <v>49.17850215261225</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>12.0864984372529</v>
+        <v>12.08649856587142</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>2.843174125611132</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.6309039658386086</v>
+        <v>0.6309039657424731</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>37.76981990394992</v>
+        <v>37.76981994446616</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>44.69111770174517</v>
+        <v>44.69111769265853</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.60604405704528</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.45626419503292</v>
+        <v>42.45626429900301</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>7.451345563806206</v>
+        <v>7.451345569956971</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.404851208806044</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.0262529236567861</v>
+        <v>0.0262529235245992</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>47.8451864598563</v>
+        <v>47.84518661879786</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>16.25201726184503</v>
+        <v>16.25201731531014</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.5521769092702236</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0257160514733801</v>
+        <v>0.0257160514517489</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>47.59182484867856</v>
+        <v>47.59182501661913</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.19533319307575</v>
+        <v>17.19533311254758</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>1.549499806986276</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0111376483528729</v>
+        <v>-0.0111376484009427</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>330.3265993024744</v>
+        <v>330.3265993024749</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>15.5</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>42.90634034065227</v>
+        <v>42.90634108900716</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>29.92037923763041</v>
+        <v>29.92037929019337</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.8504916453145873</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.008390051400245801</v>
+        <v>0.008390051316125399</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>37.02423556803554</v>
+        <v>37.02423565399497</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>14.62311298903437</v>
+        <v>14.6231130367819</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.3631057427600774</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1495860326507063</v>
+        <v>-0.1495860327107945</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>323.5728993805008</v>
+        <v>323.5728993805014</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>106</v>
@@ -6491,7 +6491,7 @@
         <v>46.91375726565757</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>13.60020483193278</v>
+        <v>13.6002048881888</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6033276840107226</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.1496197054209423</v>
+        <v>0.1496197056612832</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>321.8366154260456</v>
+        <v>321.8366154260453</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>10.3</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>40.35271489368878</v>
+        <v>40.35271501385672</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>22.18482271453169</v>
+        <v>22.18482281827115</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.302033530877532</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.0316911939716524</v>
+        <v>0.0316911939476166</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>49.85804039530499</v>
+        <v>49.85804042432328</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>5.420944955455655</v>
+        <v>5.420945098893156</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>1.204867066630291</v>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>316.5755461598397</v>
+        <v>316.575546159839</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>45</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>32.45715785282638</v>
+        <v>32.45715803087245</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>9.920301806003112</v>
+        <v>9.920301916674344</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.544182387308126</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.014265904372592</v>
+        <v>-0.0142659047090747</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>29.51377555307894</v>
+        <v>29.5137756289913</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>40.72929530895199</v>
+        <v>40.72929540335323</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.5792574912973625</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>51.02035355417789</v>
+        <v>51.0203535657951</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>7.642725548258183</v>
+        <v>7.642725563421148</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>4.144638145983135</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.1845392156606524</v>
+        <v>0.1845392156366179</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>47.52359181563961</v>
+        <v>47.52359191949896</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>8.463967369708</v>
+        <v>8.463967359141668</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1.0911250554909</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.0468111454624635</v>
+        <v>0.046811145318256</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>289.9774142795346</v>
+        <v>289.9774142795353</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>29.4</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>32.48441271570184</v>
+        <v>32.48441254376353</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>12.78322044937705</v>
+        <v>12.78322044243469</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>2.075142332672741</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.011935897973775</v>
+        <v>-0.0119358978536032</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>34.91349831782655</v>
+        <v>34.91349840067811</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>7.333365042674252</v>
+        <v>7.333365104290094</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.367877952922828</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0123972973502005</v>
+        <v>-0.0123972973622185</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>50.73375648700717</v>
+        <v>50.73375659127374</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>8.823057018978375</v>
+        <v>8.823058693391577</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.6876643918846167</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.7715169090286658</v>
+        <v>-0.7715169109831462</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>36.46194286329051</v>
+        <v>36.46194294665065</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>16.98606891657773</v>
+        <v>16.98606897652656</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.9531094343344676</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.0049703950944206</v>
+        <v>-0.0049703951785405</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>259.9033051438817</v>
+        <v>259.9033051438802</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>19.9</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>50.25244244585871</v>
+        <v>50.25244245521712</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>14.36780751475257</v>
+        <v>14.36780765906749</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>2.989079615988356</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.34079369406307</v>
+        <v>0.3407936939669274</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>44.21668250822204</v>
+        <v>44.21668251382783</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>24.00140316266452</v>
+        <v>24.0014032001776</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>1.014920947127887</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.1495503921814205</v>
+        <v>-0.1495503922054554</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>249.5903435725764</v>
+        <v>249.5903435725761</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>18.7</v>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>32.77281767285736</v>
+        <v>32.77281810184544</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>10.77934910446431</v>
+        <v>10.77934926543911</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>1.25348016857025</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0472558432708549</v>
+        <v>-0.0472558434270792</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>249.2272228586091</v>
+        <v>249.2272228586102</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>9.199999999999999</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>37.33163545238022</v>
+        <v>37.33163561589684</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>11.58467121721089</v>
+        <v>11.58467110765225</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.6137043444747197</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.0087899227677814</v>
+        <v>-0.0087899228398855</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>42.26340773041624</v>
+        <v>42.26340802580637</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>12.87277219494976</v>
+        <v>12.87277219477112</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>1.236825853447604</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.023492994732466</v>
+        <v>-0.0234929947565009</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>39.53184114054054</v>
+        <v>39.5318410446482</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>15.0527508980517</v>
+        <v>15.05275105225604</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.6475953337368624</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>0.0153591739704115</v>
+        <v>0.0153591740304993</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>44.72915647111009</v>
+        <v>44.72915651869842</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>19.08187406814932</v>
+        <v>19.08187408572832</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.8326769016424189</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>-0.0148525888817374</v>
+        <v>-0.0148525888937545</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>150.9672930010761</v>
+        <v>150.967293001076</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>15.2</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>38.89883824210713</v>
+        <v>38.89883839074079</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>18.80929684776476</v>
+        <v>18.80929678975555</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>0.4652963344820632</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.0379947148365745</v>
+        <v>0.037994714644299</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>42.33678102291245</v>
+        <v>42.33678119877486</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>16.89111736431942</v>
+        <v>16.89111742668678</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>1.037410508108879</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>0.1003077359410763</v>
+        <v>0.1003077356286301</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>

</xml_diff>